<commit_message>
fix(fixtures/claude): correct field types + remove dead fields in 4 claude patterns
- 06_merged_cells: item.price integer→currency (prices are floats like 29.99)
- 07_timesheet: line.hours integer→number (hours can be fractional like 7.5)
- 16_bundesliga: match.date datetime→string (cells are date ranges like '23./24.08.2025')
- 20_sales_report: remove dead lbl: filter_note (defined but never used in START:)

Root cause: type mismatches were causing false validation warnings. The engine's
validate_type() rejects float values for integer fields and string values for
datetime fields. Changing to the correct types eliminates 299 spurious warnings
(296 for bundesliga, 2 for timesheet, 1 for merged_cells).

Sweep improved: 23→24 clean variants, 26→25 warned, 0 errors (49 total).
1564 tests pass.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K6EyxWBecbqyp9uRx7c4J8
</commit_message>
<xml_diff>
--- a/tests/fixtures/20_sales_report/20_sales_report_pattern-from-claude.xlsx
+++ b/tests/fixtures/20_sales_report/20_sales_report_pattern-from-claude.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -526,7 +526,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>filter_note</t>
+          <t>col_product</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -536,7 +536,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Diese PivotTable wird nach den 10 meistverkauften Produkten im 1. Quartal gefiltert</t>
+          <t>Produkt</t>
         </is>
       </c>
       <c r="E4" s="2" t="n"/>
@@ -551,7 +551,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>col_product</t>
+          <t>col_q1</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -561,7 +561,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Produkt</t>
+          <t>Summe aus Qrtl 1</t>
         </is>
       </c>
       <c r="E5" s="2" t="n"/>
@@ -576,7 +576,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>col_q1</t>
+          <t>col_q2</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -586,7 +586,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Summe aus Qrtl 1</t>
+          <t>Summe aus Qrtl 2</t>
         </is>
       </c>
       <c r="E6" s="2" t="n"/>
@@ -601,7 +601,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>col_q2</t>
+          <t>col_q3</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -611,7 +611,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Summe aus Qrtl 2</t>
+          <t>Summe aus Qrtl 3</t>
         </is>
       </c>
       <c r="E7" s="2" t="n"/>
@@ -626,7 +626,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>col_q3</t>
+          <t>col_q4</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -636,7 +636,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Summe aus Qrtl 3</t>
+          <t>Summe aus Qrtl 4</t>
         </is>
       </c>
       <c r="E8" s="2" t="n"/>
@@ -644,29 +644,29 @@
       <c r="G8" s="2" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>lbl:</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>col_q4</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>var:</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>line.product</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>Summe aus Qrtl 4</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="n"/>
-      <c r="F9" s="2" t="n"/>
-      <c r="G9" s="2" t="n"/>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>.*</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="n"/>
+      <c r="F9" s="3" t="n"/>
+      <c r="G9" s="3" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -676,19 +676,15 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>line.product</t>
+          <t>line.q1</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>.*</t>
-        </is>
-      </c>
+          <t>currency</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="n"/>
       <c r="E10" s="3" t="n"/>
       <c r="F10" s="3" t="n"/>
       <c r="G10" s="3" t="n"/>
@@ -701,7 +697,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>line.q1</t>
+          <t>line.q2</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -722,7 +718,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>line.q2</t>
+          <t>line.q3</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -743,7 +739,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>line.q3</t>
+          <t>line.q4</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -757,130 +753,109 @@
       <c r="G13" s="3" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>var:</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>START:</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="n"/>
+      <c r="C14" s="4" t="n"/>
+      <c r="D14" s="4" t="n"/>
+      <c r="E14" s="4" t="n"/>
+      <c r="F14" s="4" t="n"/>
+      <c r="G14" s="4" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>table:*</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n"/>
+      <c r="C15" s="5" t="n"/>
+      <c r="D15" s="5" t="n"/>
+      <c r="E15" s="5" t="n"/>
+      <c r="F15" s="5" t="n"/>
+      <c r="G15" s="5" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n"/>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>HEADER:1</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>col_product</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>col_q1</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>col_q2</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>col_q3</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>col_q4</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="n"/>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>DATA:*</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>line.product</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>line.q1</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>line.q2</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>line.q3</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
         <is>
           <t>line.q4</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>currency</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="n"/>
-      <c r="E14" s="3" t="n"/>
-      <c r="F14" s="3" t="n"/>
-      <c r="G14" s="3" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>START:</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="n"/>
-      <c r="C15" s="4" t="n"/>
-      <c r="D15" s="4" t="n"/>
-      <c r="E15" s="4" t="n"/>
-      <c r="F15" s="4" t="n"/>
-      <c r="G15" s="4" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>table:*</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="n"/>
-      <c r="C16" s="5" t="n"/>
-      <c r="D16" s="5" t="n"/>
-      <c r="E16" s="5" t="n"/>
-      <c r="F16" s="5" t="n"/>
-      <c r="G16" s="5" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="n"/>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>HEADER:1</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>col_product</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>col_q1</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>col_q2</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>col_q3</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>col_q4</t>
-        </is>
-      </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="n"/>
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>DATA:*</t>
-        </is>
-      </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>line.product</t>
-        </is>
-      </c>
-      <c r="D18" s="3" t="inlineStr">
-        <is>
-          <t>line.q1</t>
-        </is>
-      </c>
-      <c r="E18" s="3" t="inlineStr">
-        <is>
-          <t>line.q2</t>
-        </is>
-      </c>
-      <c r="F18" s="3" t="inlineStr">
-        <is>
-          <t>line.q3</t>
-        </is>
-      </c>
-      <c r="G18" s="3" t="inlineStr">
-        <is>
-          <t>line.q4</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>END:</t>
         </is>
       </c>
-      <c r="B19" s="4" t="n"/>
-      <c r="C19" s="4" t="n"/>
-      <c r="D19" s="4" t="n"/>
-      <c r="E19" s="4" t="n"/>
-      <c r="F19" s="4" t="n"/>
-      <c r="G19" s="4" t="n"/>
+      <c r="B18" s="4" t="n"/>
+      <c r="C18" s="4" t="n"/>
+      <c r="D18" s="4" t="n"/>
+      <c r="E18" s="4" t="n"/>
+      <c r="F18" s="4" t="n"/>
+      <c r="G18" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>